<commit_message>
Compare Age 18-24 vs 25-35 research segments on the dashboard and in Ask AI.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Myntra Wishlist.xlsx
+++ b/Myntra Wishlist.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\smustafi\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E5D9CC69-D312-46E5-8415-726E6614A830}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66CB43DD-78CF-41CC-8255-82A14363B718}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="69">
   <si>
     <t>Timestamp</t>
   </si>
@@ -319,6 +319,12 @@
   </si>
   <si>
     <t>Clothing, Accessories</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Age </t>
+  </si>
+  <si>
+    <t>25-35</t>
   </si>
 </sst>
 </file>
@@ -398,22 +404,24 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="5">
     <dxf>
-      <border>
-        <left style="thin">
-          <color rgb="FF5B3F86"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF5B3F86"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF5B3F86"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF5B3F86"/>
-        </bottom>
-      </border>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <fill>
@@ -439,10 +447,26 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color rgb="FF5B3F86"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF5B3F86"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF5B3F86"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF5B3F86"/>
+        </bottom>
+      </border>
+    </dxf>
   </dxfs>
   <tableStyles count="1">
     <tableStyle name="Form responses 1-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="0"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="4"/>
       <tableStyleElement type="headerRow" dxfId="3"/>
       <tableStyleElement type="firstRowStripe" dxfId="2"/>
       <tableStyleElement type="secondRowStripe" dxfId="1"/>
@@ -460,12 +484,13 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Form_Responses" displayName="Form_Responses" ref="A1:S10">
-  <tableColumns count="19">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Form_Responses" displayName="Form_Responses" ref="A1:T10">
+  <tableColumns count="20">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Timestamp"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="1. Do you currently use Myntra?"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="2. Have you used Myntra’s wishlist feature?"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="3. How often do you add items to your Myntra wishlist?"/>
+    <tableColumn id="20" xr3:uid="{3F0A037C-7E8F-4128-A4EF-A7277AFCEDAF}" name="Age " dataDxfId="0"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="4. Approximately how many items are currently in your wishlist?"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="5. What types of products do you usually save?"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="6. How long do you usually keep items in your wishlist before deciding what to do?"/>
@@ -687,16 +712,16 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:S10"/>
+  <dimension ref="A1:T10"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.90625" customWidth="1"/>
     <col min="2" max="2" width="29.36328125" customWidth="1"/>
-    <col min="3" max="19" width="37.6328125" customWidth="1"/>
-    <col min="20" max="25" width="18.90625" customWidth="1"/>
+    <col min="3" max="20" width="37.6328125" customWidth="1"/>
+    <col min="21" max="26" width="18.90625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -710,52 +735,55 @@
         <v>3</v>
       </c>
       <c r="E1" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="S1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="2" t="s">
+      <c r="T1" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:19" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:20" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>46255.761461909722</v>
       </c>
@@ -769,34 +797,34 @@
         <v>21</v>
       </c>
       <c r="E2" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="F2" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="G2" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="H2" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="I2" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="J2" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="K2" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="K2" s="4" t="s">
+      <c r="L2" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="L2" s="4" t="s">
+      <c r="M2" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="M2" s="4" t="s">
+      <c r="N2" s="4" t="s">
         <v>30</v>
-      </c>
-      <c r="N2" s="4" t="s">
-        <v>29</v>
       </c>
       <c r="O2" s="4" t="s">
         <v>29</v>
@@ -808,11 +836,14 @@
         <v>29</v>
       </c>
       <c r="R2" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="S2" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="S2" s="4"/>
+      <c r="T2" s="4"/>
     </row>
-    <row r="3" spans="1:19" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:20" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>46255.764285324069</v>
       </c>
@@ -826,46 +857,49 @@
         <v>34</v>
       </c>
       <c r="E3" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="F3" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="G3" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="H3" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="I3" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="I3" s="4" t="s">
+      <c r="J3" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="J3" s="4" t="s">
+      <c r="K3" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="K3" s="4" t="s">
+      <c r="L3" s="4" t="s">
         <v>40</v>
-      </c>
-      <c r="L3" s="4" t="s">
-        <v>29</v>
       </c>
       <c r="M3" s="4" t="s">
         <v>29</v>
       </c>
       <c r="N3" s="4" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="O3" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="P3" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="P3" s="4" t="s">
+      <c r="Q3" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="Q3" s="4" t="s">
+      <c r="R3" s="4" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="4" spans="1:19" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:20" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>46255.799973356479</v>
       </c>
@@ -879,46 +913,49 @@
         <v>34</v>
       </c>
       <c r="E4" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="F4" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="G4" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="H4" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="H4" s="4" t="s">
+      <c r="I4" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="I4" s="4" t="s">
+      <c r="J4" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="J4" s="4" t="s">
+      <c r="K4" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="K4" s="4" t="s">
+      <c r="L4" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="L4" s="4" t="s">
-        <v>41</v>
-      </c>
       <c r="M4" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="N4" s="4" t="s">
         <v>29</v>
-      </c>
-      <c r="N4" s="4" t="s">
-        <v>42</v>
       </c>
       <c r="O4" s="4" t="s">
         <v>42</v>
       </c>
       <c r="P4" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="Q4" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="Q4" s="4" t="s">
+      <c r="R4" s="4" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="5" spans="1:19" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:20" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>46255.823812708331</v>
       </c>
@@ -932,46 +969,49 @@
         <v>34</v>
       </c>
       <c r="E5" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="F5" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="G5" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="H5" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="I5" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="I5" s="4" t="s">
+      <c r="J5" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="J5" s="4" t="s">
+      <c r="K5" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="K5" s="4" t="s">
+      <c r="L5" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="L5" s="4" t="s">
+      <c r="M5" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="M5" s="4" t="s">
-        <v>41</v>
-      </c>
       <c r="N5" s="4" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="O5" s="4" t="s">
         <v>29</v>
       </c>
       <c r="P5" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q5" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="Q5" s="4" t="s">
+      <c r="R5" s="4" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="6" spans="1:19" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:20" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>46255.911578634259</v>
       </c>
@@ -985,46 +1025,49 @@
         <v>34</v>
       </c>
       <c r="E6" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="F6" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="G6" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="H6" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="I6" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="I6" s="4" t="s">
+      <c r="J6" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="J6" s="4" t="s">
+      <c r="K6" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="K6" s="4" t="s">
+      <c r="L6" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="L6" s="4" t="s">
+      <c r="M6" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="M6" s="4" t="s">
-        <v>41</v>
-      </c>
       <c r="N6" s="4" t="s">
         <v>41</v>
       </c>
       <c r="O6" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="P6" s="4" t="s">
         <v>47</v>
-      </c>
-      <c r="P6" s="4" t="s">
-        <v>42</v>
       </c>
       <c r="Q6" s="4" t="s">
         <v>42</v>
       </c>
+      <c r="R6" s="4" t="s">
+        <v>42</v>
+      </c>
     </row>
-    <row r="7" spans="1:19" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:20" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>46256.030755532411</v>
       </c>
@@ -1038,46 +1081,49 @@
         <v>34</v>
       </c>
       <c r="E7" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="F7" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="G7" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="G7" s="4" t="s">
+      <c r="H7" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="H7" s="4" t="s">
+      <c r="I7" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="I7" s="4" t="s">
+      <c r="J7" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="J7" s="4" t="s">
+      <c r="K7" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="K7" s="4" t="s">
+      <c r="L7" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="L7" s="4" t="s">
+      <c r="M7" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="M7" s="4" t="s">
-        <v>41</v>
-      </c>
       <c r="N7" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="O7" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="O7" s="4" t="s">
-        <v>41</v>
-      </c>
       <c r="P7" s="4" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="Q7" s="4" t="s">
         <v>29</v>
       </c>
+      <c r="R7" s="4" t="s">
+        <v>29</v>
+      </c>
     </row>
-    <row r="8" spans="1:19" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:20" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>46256.592458726853</v>
       </c>
@@ -1091,34 +1137,34 @@
         <v>34</v>
       </c>
       <c r="E8" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="F8" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="G8" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="G8" s="4" t="s">
+      <c r="H8" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="H8" s="4" t="s">
+      <c r="I8" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="I8" s="4" t="s">
+      <c r="J8" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="J8" s="4" t="s">
+      <c r="K8" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="K8" s="4" t="s">
+      <c r="L8" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="L8" s="4" t="s">
+      <c r="M8" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="M8" s="4" t="s">
-        <v>41</v>
-      </c>
       <c r="N8" s="4" t="s">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="O8" s="4" t="s">
         <v>30</v>
@@ -1130,13 +1176,16 @@
         <v>30</v>
       </c>
       <c r="R8" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="S8" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="S8" s="4" t="s">
+      <c r="T8" s="4" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="9" spans="1:19" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:20" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
         <v>46256.616355706021</v>
       </c>
@@ -1150,52 +1199,55 @@
         <v>34</v>
       </c>
       <c r="E9" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="F9" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="F9" s="4" t="s">
+      <c r="G9" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="G9" s="4" t="s">
+      <c r="H9" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="H9" s="4" t="s">
+      <c r="I9" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="I9" s="4" t="s">
+      <c r="J9" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="J9" s="4" t="s">
+      <c r="K9" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="K9" s="4" t="s">
+      <c r="L9" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="L9" s="4" t="s">
+      <c r="M9" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="M9" s="4" t="s">
-        <v>41</v>
-      </c>
       <c r="N9" s="4" t="s">
         <v>41</v>
       </c>
       <c r="O9" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="P9" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="P9" s="4" t="s">
-        <v>41</v>
-      </c>
       <c r="Q9" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="R9" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="R9" s="4" t="s">
+      <c r="S9" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="S9" s="4" t="s">
+      <c r="T9" s="4" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="10" spans="1:19" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:20" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3">
         <v>46256.644537905093</v>
       </c>
@@ -1209,29 +1261,29 @@
         <v>34</v>
       </c>
       <c r="E10" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="F10" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="F10" s="4" t="s">
+      <c r="G10" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="G10" s="4" t="s">
+      <c r="H10" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="H10" s="4" t="s">
+      <c r="I10" s="4" t="s">
         <v>37</v>
-      </c>
-      <c r="I10" s="4" t="s">
-        <v>58</v>
       </c>
       <c r="J10" s="4" t="s">
         <v>58</v>
       </c>
       <c r="K10" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="L10" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="L10" s="4" t="s">
-        <v>41</v>
-      </c>
       <c r="M10" s="4" t="s">
         <v>41</v>
       </c>
@@ -1245,6 +1297,9 @@
         <v>41</v>
       </c>
       <c r="Q10" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="R10" s="4" t="s">
         <v>41</v>
       </c>
     </row>
@@ -1257,6 +1312,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101001DC02A62EFC9634297276F9F40B9E4BD" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="fcaf9f9ad54ec0105f14d00ed35c9a49">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="f06966d8-1906-449d-9f16-0f9261b83eb0" xmlns:ns4="0e3235cb-450d-405b-957b-f9dc6b0fe889" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="53ba5807e3e26b58aa3af9af24d73626" ns3:_="" ns4:_="">
     <xsd:import namespace="f06966d8-1906-449d-9f16-0f9261b83eb0"/>
@@ -1497,15 +1561,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -1515,6 +1570,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{63595264-DBEF-41B7-9171-2ABE3CA10C3F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B235B7D7-E070-4754-9957-658C0CF4EEFA}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1529,14 +1592,6 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{63595264-DBEF-41B7-9171-2ABE3CA10C3F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>